<commit_message>
Added correction functions and stuf (67)
</commit_message>
<xml_diff>
--- a/CORRECTIONS_V2/CORRECTIONS_SHEET.xlsx
+++ b/CORRECTIONS_V2/CORRECTIONS_SHEET.xlsx
@@ -5,22 +5,23 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\douwe\AE4115-23_EXPERIMENTAL SIMULATIONS\Group_15_Redo_BAL\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\douwe\AE4115-23_EXPERIMENTAL SIMULATIONS\Group_15_Redo_BAL\CORRECTIONS_V2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63A8D540-164E-4E3F-BA77-18C4C817EFD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF75C0B0-C47C-4CC2-B12D-76BD2E8A3F07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="1605" windowWidth="29040" windowHeight="15720" xr2:uid="{6779DE78-6A77-4C37-B946-ECD2BA7E5752}"/>
+    <workbookView xWindow="3864" yWindow="2040" windowWidth="17280" windowHeight="9960" activeTab="3" xr2:uid="{6779DE78-6A77-4C37-B946-ECD2BA7E5752}"/>
   </bookViews>
   <sheets>
     <sheet name="solid_body_blockage" sheetId="1" r:id="rId1"/>
     <sheet name="PROP" sheetId="2" r:id="rId2"/>
     <sheet name="WING" sheetId="4" r:id="rId3"/>
-    <sheet name="FUSELAGE" sheetId="5" r:id="rId4"/>
-    <sheet name="HORIZONTAL_TAIL" sheetId="6" r:id="rId5"/>
-    <sheet name="VERTICAL_TAIL" sheetId="7" r:id="rId6"/>
-    <sheet name="TUNNEL" sheetId="8" r:id="rId7"/>
-    <sheet name="STRUTS" sheetId="9" r:id="rId8"/>
+    <sheet name="tail_correction" sheetId="10" r:id="rId4"/>
+    <sheet name="FUSELAGE" sheetId="5" r:id="rId5"/>
+    <sheet name="HORIZONTAL_TAIL" sheetId="6" r:id="rId6"/>
+    <sheet name="VERTICAL_TAIL" sheetId="7" r:id="rId7"/>
+    <sheet name="TUNNEL" sheetId="8" r:id="rId8"/>
+    <sheet name="STRUTS" sheetId="9" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="174">
   <si>
     <t>Body</t>
   </si>
@@ -526,6 +527,45 @@
   </si>
   <si>
     <t>Values used in solid blockage calculations</t>
+  </si>
+  <si>
+    <t>Final TailOff</t>
+  </si>
+  <si>
+    <t>AR_wing</t>
+  </si>
+  <si>
+    <t>S_wing</t>
+  </si>
+  <si>
+    <t>MAC_wing</t>
+  </si>
+  <si>
+    <t>AR_tail</t>
+  </si>
+  <si>
+    <t>S_tail</t>
+  </si>
+  <si>
+    <t>Length_tail</t>
+  </si>
+  <si>
+    <t>Wing</t>
+  </si>
+  <si>
+    <t>Tail</t>
+  </si>
+  <si>
+    <t>[m^2]</t>
+  </si>
+  <si>
+    <t>[m]</t>
+  </si>
+  <si>
+    <t>(q_t/q)* a_t</t>
+  </si>
+  <si>
+    <t>dCm_0.25c / da_t</t>
   </si>
 </sst>
 </file>
@@ -534,7 +574,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="170" formatCode="0.0000"/>
+    <numFmt numFmtId="164" formatCode="0.0000"/>
   </numFmts>
   <fonts count="5" x14ac:knownFonts="1">
     <font>
@@ -575,7 +615,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -630,8 +670,20 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.749992370372631"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="40">
+  <borders count="45">
     <border>
       <left/>
       <right/>
@@ -1142,6 +1194,77 @@
         <color indexed="64"/>
       </top>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="double">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -1159,32 +1282,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -1217,31 +1324,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -1263,47 +1345,94 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="39" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="31" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="39" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="31" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="32" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="42" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="44" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -2016,136 +2145,136 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="84" t="s">
+      <c r="A1" s="65" t="s">
         <v>160</v>
       </c>
-      <c r="B1" s="83"/>
-      <c r="C1" s="83"/>
-      <c r="D1" s="83"/>
-      <c r="E1" s="83"/>
-      <c r="F1" s="83"/>
-      <c r="G1" s="83"/>
-      <c r="H1" s="83"/>
-      <c r="I1" s="83"/>
-      <c r="J1" s="83"/>
-      <c r="K1" s="83"/>
-      <c r="L1" s="83"/>
-      <c r="M1" s="83"/>
-      <c r="N1" s="83"/>
-      <c r="O1" s="83"/>
+      <c r="B1" s="66"/>
+      <c r="C1" s="66"/>
+      <c r="D1" s="66"/>
+      <c r="E1" s="66"/>
+      <c r="F1" s="66"/>
+      <c r="G1" s="66"/>
+      <c r="H1" s="66"/>
+      <c r="I1" s="66"/>
+      <c r="J1" s="66"/>
+      <c r="K1" s="66"/>
+      <c r="L1" s="66"/>
+      <c r="M1" s="66"/>
+      <c r="N1" s="66"/>
+      <c r="O1" s="66"/>
     </row>
     <row r="2" spans="1:15" ht="15.6" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="13" t="s">
+      <c r="B2" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="11" t="s">
+      <c r="C2" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="11" t="s">
+      <c r="D2" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="11" t="s">
+      <c r="E2" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="F2" s="11" t="s">
+      <c r="F2" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="G2" s="11" t="s">
+      <c r="G2" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="21" t="s">
+      <c r="H2" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="I2" s="38" t="s">
+      <c r="I2" s="30" t="s">
         <v>112</v>
       </c>
-      <c r="J2" s="48" t="s">
+      <c r="J2" s="9" t="s">
         <v>133</v>
       </c>
-      <c r="K2" s="48" t="s">
+      <c r="K2" s="9" t="s">
         <v>134</v>
       </c>
-      <c r="L2" s="48" t="s">
+      <c r="L2" s="9" t="s">
         <v>135</v>
       </c>
-      <c r="M2" s="11" t="s">
+      <c r="M2" s="9" t="s">
         <v>136</v>
       </c>
-      <c r="N2" s="60" t="s">
+      <c r="N2" s="43" t="s">
         <v>137</v>
       </c>
-      <c r="O2" s="60" t="s">
+      <c r="O2" s="43" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="3" spans="1:15" ht="15.6" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="22" t="s">
+      <c r="A3" s="75" t="s">
         <v>125</v>
       </c>
-      <c r="B3" s="22"/>
-      <c r="C3" s="22"/>
-      <c r="D3" s="22"/>
-      <c r="E3" s="22"/>
-      <c r="F3" s="22"/>
-      <c r="G3" s="22"/>
-      <c r="H3" s="22"/>
-      <c r="I3" s="46" t="s">
+      <c r="B3" s="75"/>
+      <c r="C3" s="75"/>
+      <c r="D3" s="75"/>
+      <c r="E3" s="75"/>
+      <c r="F3" s="75"/>
+      <c r="G3" s="75"/>
+      <c r="H3" s="75"/>
+      <c r="I3" s="76" t="s">
         <v>139</v>
       </c>
-      <c r="J3" s="47"/>
-      <c r="K3" s="47"/>
-      <c r="L3" s="47"/>
-      <c r="M3" s="47"/>
-      <c r="N3" s="50" t="s">
+      <c r="J3" s="77"/>
+      <c r="K3" s="77"/>
+      <c r="L3" s="77"/>
+      <c r="M3" s="77"/>
+      <c r="N3" s="69" t="s">
         <v>140</v>
       </c>
-      <c r="O3" s="49"/>
+      <c r="O3" s="71"/>
     </row>
     <row r="4" spans="1:15" ht="15" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="16" t="s">
+      <c r="A4" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="14">
+      <c r="B4" s="12">
         <v>3.0228999999999998E-3</v>
       </c>
       <c r="C4" s="2">
         <v>1.397</v>
       </c>
-      <c r="D4" s="27" t="s">
+      <c r="D4" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="E4" s="27" t="s">
+      <c r="E4" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="F4" s="10">
+      <c r="F4" s="2">
         <v>0.2172</v>
       </c>
-      <c r="G4" s="10">
+      <c r="G4" s="2">
         <v>0.16500000000000001</v>
       </c>
-      <c r="H4" s="34" t="s">
+      <c r="H4" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="I4" s="41">
+      <c r="I4" s="33">
         <v>0.15</v>
       </c>
-      <c r="J4" s="27" t="s">
+      <c r="J4" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="K4" s="52">
+      <c r="K4" s="35">
         <v>64</v>
       </c>
-      <c r="L4" s="63">
+      <c r="L4" s="46">
         <f>C4/$B$19</f>
         <v>0.77611111111111108</v>
       </c>
-      <c r="M4" s="55">
+      <c r="M4" s="38">
         <v>1.43</v>
       </c>
-      <c r="N4" s="58">
+      <c r="N4" s="41">
         <v>1.02</v>
       </c>
       <c r="O4" s="2">
@@ -2153,7 +2282,7 @@
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A5" s="17" t="s">
+      <c r="A5" s="14" t="s">
         <v>3</v>
       </c>
       <c r="B5" s="3">
@@ -2162,10 +2291,10 @@
       <c r="C5" s="1">
         <v>0.57599999999999996</v>
       </c>
-      <c r="D5" s="28" t="s">
+      <c r="D5" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="E5" s="28" t="s">
+      <c r="E5" s="20" t="s">
         <v>16</v>
       </c>
       <c r="F5" s="1">
@@ -2174,26 +2303,26 @@
       <c r="G5" s="1">
         <v>0.14899999999999999</v>
       </c>
-      <c r="H5" s="35" t="s">
+      <c r="H5" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="I5" s="39">
+      <c r="I5" s="31">
         <v>0.15</v>
       </c>
-      <c r="J5" s="28" t="s">
+      <c r="J5" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="K5" s="40">
+      <c r="K5" s="32">
         <v>64</v>
       </c>
       <c r="L5" s="2">
-        <f t="shared" ref="L5:L6" si="0">C5/$B$19</f>
+        <f t="shared" ref="L5" si="0">C5/$B$19</f>
         <v>0.31999999999999995</v>
       </c>
-      <c r="M5" s="56">
+      <c r="M5" s="39">
         <v>1.43</v>
       </c>
-      <c r="N5" s="37">
+      <c r="N5" s="29">
         <v>1.02</v>
       </c>
       <c r="O5" s="1">
@@ -2201,7 +2330,7 @@
       </c>
     </row>
     <row r="6" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="19" t="s">
+      <c r="A6" s="16" t="s">
         <v>4</v>
       </c>
       <c r="B6" s="5">
@@ -2210,10 +2339,10 @@
       <c r="C6" s="7">
         <v>0.25800000000000001</v>
       </c>
-      <c r="D6" s="29" t="s">
+      <c r="D6" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="E6" s="29" t="s">
+      <c r="E6" s="21" t="s">
         <v>16</v>
       </c>
       <c r="F6" s="7">
@@ -2222,26 +2351,26 @@
       <c r="G6" s="7">
         <v>0.17</v>
       </c>
-      <c r="H6" s="36" t="s">
+      <c r="H6" s="28" t="s">
         <v>18</v>
       </c>
-      <c r="I6" s="42">
+      <c r="I6" s="34">
         <v>0.15</v>
       </c>
-      <c r="J6" s="29" t="s">
+      <c r="J6" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="K6" s="53" t="s">
+      <c r="K6" s="36" t="s">
         <v>141</v>
       </c>
-      <c r="L6" s="63">
+      <c r="L6" s="46">
         <f>C6/$B$19</f>
         <v>0.14333333333333334</v>
       </c>
-      <c r="M6" s="57">
+      <c r="M6" s="40">
         <v>1.43</v>
       </c>
-      <c r="N6" s="59">
+      <c r="N6" s="42">
         <v>1.03833</v>
       </c>
       <c r="O6" s="7">
@@ -2249,36 +2378,36 @@
       </c>
     </row>
     <row r="7" spans="1:15" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="23" t="s">
+      <c r="A7" s="74" t="s">
         <v>123</v>
       </c>
-      <c r="B7" s="22"/>
-      <c r="C7" s="22"/>
-      <c r="D7" s="22"/>
-      <c r="E7" s="22"/>
-      <c r="F7" s="22"/>
-      <c r="G7" s="22"/>
-      <c r="H7" s="22"/>
-      <c r="I7" s="45" t="s">
+      <c r="B7" s="75"/>
+      <c r="C7" s="75"/>
+      <c r="D7" s="75"/>
+      <c r="E7" s="75"/>
+      <c r="F7" s="75"/>
+      <c r="G7" s="75"/>
+      <c r="H7" s="75"/>
+      <c r="I7" s="67" t="s">
         <v>139</v>
       </c>
-      <c r="J7" s="44"/>
-      <c r="K7" s="44"/>
-      <c r="L7" s="44"/>
-      <c r="M7" s="44"/>
-      <c r="N7" s="50" t="s">
+      <c r="J7" s="78"/>
+      <c r="K7" s="78"/>
+      <c r="L7" s="78"/>
+      <c r="M7" s="78"/>
+      <c r="N7" s="69" t="s">
         <v>140</v>
       </c>
-      <c r="O7" s="51"/>
+      <c r="O7" s="70"/>
     </row>
     <row r="8" spans="1:15" ht="15" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="16" t="s">
+      <c r="A8" s="13" t="s">
         <v>2</v>
       </c>
       <c r="B8" s="4">
         <v>1.60632E-2</v>
       </c>
-      <c r="C8" s="27" t="s">
+      <c r="C8" s="19" t="s">
         <v>16</v>
       </c>
       <c r="D8" s="2">
@@ -2287,32 +2416,32 @@
       <c r="E8" s="2">
         <v>0.14000000000000001</v>
       </c>
-      <c r="F8" s="27" t="s">
+      <c r="F8" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="G8" s="27" t="s">
+      <c r="G8" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="H8" s="32" t="s">
+      <c r="H8" s="24" t="s">
         <v>16</v>
       </c>
-      <c r="I8" s="62" t="s">
+      <c r="I8" s="45" t="s">
         <v>16</v>
       </c>
-      <c r="J8" s="64">
+      <c r="J8" s="47">
         <f>E8/D8</f>
         <v>0.10432190760059613</v>
       </c>
-      <c r="K8" s="54" t="s">
+      <c r="K8" s="37" t="s">
         <v>142</v>
       </c>
       <c r="L8" s="2">
         <v>0</v>
       </c>
-      <c r="M8" s="55">
+      <c r="M8" s="38">
         <v>1.43</v>
       </c>
-      <c r="N8" s="58">
+      <c r="N8" s="41">
         <v>0.91</v>
       </c>
       <c r="O8" s="2">
@@ -2320,13 +2449,13 @@
       </c>
     </row>
     <row r="9" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="19" t="s">
+      <c r="A9" s="16" t="s">
         <v>156</v>
       </c>
       <c r="B9" s="5">
         <v>7.9210000000000001E-4</v>
       </c>
-      <c r="C9" s="29" t="s">
+      <c r="C9" s="21" t="s">
         <v>16</v>
       </c>
       <c r="D9" s="7">
@@ -2336,32 +2465,32 @@
         <f>0.28*0.2032</f>
         <v>5.6896000000000002E-2</v>
       </c>
-      <c r="F9" s="29" t="s">
+      <c r="F9" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="G9" s="29" t="s">
+      <c r="G9" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="H9" s="33" t="s">
+      <c r="H9" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="I9" s="61" t="s">
+      <c r="I9" s="44" t="s">
         <v>16</v>
       </c>
-      <c r="J9" s="63">
+      <c r="J9" s="46">
         <f>E9/D9</f>
         <v>0.16491594202898552</v>
       </c>
-      <c r="K9" s="53" t="s">
+      <c r="K9" s="36" t="s">
         <v>142</v>
       </c>
       <c r="L9" s="7">
         <v>0</v>
       </c>
-      <c r="M9" s="57">
+      <c r="M9" s="40">
         <v>1.43</v>
       </c>
-      <c r="N9" s="59">
+      <c r="N9" s="42">
         <v>0.93330000000000002</v>
       </c>
       <c r="O9" s="7">
@@ -2369,30 +2498,30 @@
       </c>
     </row>
     <row r="10" spans="1:15" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="23" t="s">
+      <c r="A10" s="74" t="s">
         <v>124</v>
       </c>
-      <c r="B10" s="22"/>
-      <c r="C10" s="22"/>
-      <c r="D10" s="22"/>
-      <c r="E10" s="22"/>
-      <c r="F10" s="22"/>
-      <c r="G10" s="22"/>
-      <c r="H10" s="22"/>
-      <c r="I10" s="45" t="s">
+      <c r="B10" s="75"/>
+      <c r="C10" s="75"/>
+      <c r="D10" s="75"/>
+      <c r="E10" s="75"/>
+      <c r="F10" s="75"/>
+      <c r="G10" s="75"/>
+      <c r="H10" s="75"/>
+      <c r="I10" s="67" t="s">
         <v>139</v>
       </c>
-      <c r="J10" s="43"/>
-      <c r="K10" s="43"/>
-      <c r="L10" s="43"/>
-      <c r="M10" s="43"/>
-      <c r="N10" s="50" t="s">
+      <c r="J10" s="68"/>
+      <c r="K10" s="68"/>
+      <c r="L10" s="68"/>
+      <c r="M10" s="68"/>
+      <c r="N10" s="69" t="s">
         <v>140</v>
       </c>
-      <c r="O10" s="51"/>
+      <c r="O10" s="70"/>
     </row>
     <row r="11" spans="1:15" ht="15" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="16" t="s">
+      <c r="A11" s="13" t="s">
         <v>159</v>
       </c>
       <c r="B11" s="4">
@@ -2407,36 +2536,36 @@
         <f>J22/1000</f>
         <v>0.61</v>
       </c>
-      <c r="E11" s="27" t="s">
+      <c r="E11" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="F11" s="27" t="s">
+      <c r="F11" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="G11" s="27" t="s">
+      <c r="G11" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="H11" s="69" t="s">
+      <c r="H11" s="52" t="s">
         <v>149</v>
       </c>
-      <c r="I11" s="68">
+      <c r="I11" s="51">
         <f>J21</f>
         <v>0.2857142857142857</v>
       </c>
-      <c r="J11" s="27" t="s">
+      <c r="J11" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="K11" s="54" t="s">
+      <c r="K11" s="37" t="s">
         <v>141</v>
       </c>
-      <c r="L11" s="63">
+      <c r="L11" s="46">
         <f>D11/B19</f>
         <v>0.33888888888888885</v>
       </c>
-      <c r="M11" s="55">
+      <c r="M11" s="38">
         <v>1.43</v>
       </c>
-      <c r="N11" s="71">
+      <c r="N11" s="41">
         <v>1.1000000000000001</v>
       </c>
       <c r="O11" s="2">
@@ -2444,10 +2573,10 @@
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A12" s="17" t="s">
+      <c r="A12" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="B12" s="15">
+      <c r="B12" s="3">
         <v>4.4910000000000002E-4</v>
       </c>
       <c r="C12" s="1">
@@ -2458,85 +2587,73 @@
         <f>F22/1000</f>
         <v>0.7</v>
       </c>
-      <c r="E12" s="28" t="s">
+      <c r="E12" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="F12" s="28" t="s">
+      <c r="F12" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="G12" s="28" t="s">
+      <c r="G12" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="H12" s="70" t="s">
+      <c r="H12" s="53" t="s">
         <v>147</v>
       </c>
-      <c r="I12" s="67">
+      <c r="I12" s="50">
         <f>F21</f>
         <v>0.24915596573736898</v>
       </c>
-      <c r="J12" s="28" t="s">
+      <c r="J12" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="K12" s="65" t="s">
+      <c r="K12" s="48" t="s">
         <v>141</v>
       </c>
-      <c r="L12" s="66">
+      <c r="L12" s="49">
         <f>C12/B19</f>
         <v>0.38888888888888884</v>
       </c>
-      <c r="M12" s="56">
+      <c r="M12" s="39">
         <v>1.43</v>
       </c>
-      <c r="N12" s="72">
+      <c r="N12" s="29">
         <v>1.1000000000000001</v>
       </c>
       <c r="O12" s="1">
         <v>0.86250000000000004</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="H15" s="24"/>
-    </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="C16" s="24"/>
-      <c r="D16" s="24"/>
-      <c r="H16" s="24"/>
-    </row>
     <row r="17" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="26" t="s">
+      <c r="A17" s="72" t="s">
         <v>132</v>
       </c>
-      <c r="B17" s="25"/>
-      <c r="C17" s="25"/>
-      <c r="D17" s="24"/>
-      <c r="E17" s="26" t="s">
+      <c r="B17" s="73"/>
+      <c r="C17" s="73"/>
+      <c r="E17" s="72" t="s">
         <v>143</v>
       </c>
-      <c r="F17" s="25"/>
-      <c r="G17" s="25"/>
-      <c r="I17" s="26" t="s">
+      <c r="F17" s="73"/>
+      <c r="G17" s="73"/>
+      <c r="I17" s="72" t="s">
         <v>148</v>
       </c>
-      <c r="J17" s="25"/>
-      <c r="K17" s="25"/>
-      <c r="N17" s="24"/>
-      <c r="O17" s="24"/>
+      <c r="J17" s="73"/>
+      <c r="K17" s="73"/>
     </row>
     <row r="18" spans="1:15" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="B18" s="20" t="s">
+      <c r="B18" s="17" t="s">
         <v>21</v>
       </c>
       <c r="C18" s="8" t="s">
         <v>126</v>
       </c>
-      <c r="D18" s="24"/>
       <c r="E18" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="F18" s="20" t="s">
+      <c r="F18" s="17" t="s">
         <v>21</v>
       </c>
       <c r="G18" s="8" t="s">
@@ -2545,189 +2662,176 @@
       <c r="I18" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="J18" s="20" t="s">
+      <c r="J18" s="17" t="s">
         <v>21</v>
       </c>
       <c r="K18" s="8" t="s">
         <v>126</v>
       </c>
-      <c r="O18" s="73"/>
+      <c r="O18" s="54"/>
     </row>
     <row r="19" spans="1:15" ht="15" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="16" t="s">
+      <c r="A19" s="13" t="s">
         <v>127</v>
       </c>
       <c r="B19" s="4">
         <f>TUNNEL!B2</f>
         <v>1.8</v>
       </c>
-      <c r="C19" s="30" t="s">
+      <c r="C19" s="22" t="s">
         <v>120</v>
       </c>
-      <c r="E19" s="16" t="s">
+      <c r="E19" s="13" t="s">
         <v>144</v>
       </c>
       <c r="F19" s="4">
         <v>16.899999999999999</v>
       </c>
-      <c r="G19" s="30" t="s">
+      <c r="G19" s="22" t="s">
         <v>146</v>
       </c>
-      <c r="I19" s="16" t="s">
+      <c r="I19" s="13" t="s">
         <v>144</v>
       </c>
       <c r="J19" s="4">
         <v>20</v>
       </c>
-      <c r="K19" s="30" t="s">
+      <c r="K19" s="22" t="s">
         <v>146</v>
       </c>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A20" s="17" t="s">
+      <c r="A20" s="14" t="s">
         <v>128</v>
       </c>
       <c r="B20" s="3">
         <f>TUNNEL!B3</f>
         <v>1.25</v>
       </c>
-      <c r="C20" s="31" t="s">
+      <c r="C20" s="23" t="s">
         <v>120</v>
       </c>
-      <c r="E20" s="17" t="s">
+      <c r="E20" s="14" t="s">
         <v>145</v>
       </c>
       <c r="F20" s="3">
         <f>67.829</f>
         <v>67.828999999999994</v>
       </c>
-      <c r="G20" s="31" t="s">
+      <c r="G20" s="23" t="s">
         <v>146</v>
       </c>
-      <c r="I20" s="17" t="s">
+      <c r="I20" s="14" t="s">
         <v>145</v>
       </c>
       <c r="J20" s="3">
         <v>70</v>
       </c>
-      <c r="K20" s="31" t="s">
+      <c r="K20" s="23" t="s">
         <v>146</v>
       </c>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A21" s="17" t="s">
+      <c r="A21" s="14" t="s">
         <v>122</v>
       </c>
       <c r="B21" s="3">
         <f>TUNNEL!B8</f>
         <v>1.44</v>
       </c>
-      <c r="C21" s="31" t="s">
+      <c r="C21" s="23" t="s">
         <v>131</v>
       </c>
-      <c r="E21" s="17" t="s">
+      <c r="E21" s="14" t="s">
         <v>112</v>
       </c>
       <c r="F21" s="3">
         <f>F19/F20</f>
         <v>0.24915596573736898</v>
       </c>
-      <c r="G21" s="31" t="s">
+      <c r="G21" s="23" t="s">
         <v>131</v>
       </c>
-      <c r="I21" s="17" t="s">
+      <c r="I21" s="14" t="s">
         <v>112</v>
       </c>
       <c r="J21" s="3">
         <f>J19/J20</f>
         <v>0.2857142857142857</v>
       </c>
-      <c r="K21" s="31" t="s">
+      <c r="K21" s="23" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A22" s="17" t="s">
+      <c r="A22" s="14" t="s">
         <v>129</v>
       </c>
       <c r="B22" s="3">
         <f>TUNNEL!B7</f>
         <v>2.0699999999999998</v>
       </c>
-      <c r="C22" s="31" t="s">
+      <c r="C22" s="23" t="s">
         <v>130</v>
       </c>
-      <c r="E22" s="17" t="s">
+      <c r="E22" s="14" t="s">
         <v>8</v>
       </c>
       <c r="F22" s="3">
         <v>700</v>
       </c>
-      <c r="G22" s="31" t="s">
+      <c r="G22" s="23" t="s">
         <v>146</v>
       </c>
-      <c r="H22" s="78"/>
-      <c r="I22" s="17" t="s">
+      <c r="I22" s="14" t="s">
         <v>8</v>
       </c>
       <c r="J22" s="3">
         <v>610</v>
       </c>
-      <c r="K22" s="31" t="s">
+      <c r="K22" s="23" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="H23" s="79"/>
-    </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="E24" s="24"/>
-      <c r="F24" s="24"/>
-      <c r="G24" s="24"/>
-    </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="B25" s="24"/>
-      <c r="C25" s="24"/>
-      <c r="F25" s="80"/>
-      <c r="G25" s="79"/>
-      <c r="H25" s="78"/>
+      <c r="F25" s="59"/>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A26" s="81" t="s">
+      <c r="A26" s="63" t="s">
         <v>157</v>
       </c>
-      <c r="B26" s="82"/>
-      <c r="C26" s="82"/>
-      <c r="D26" s="82"/>
-      <c r="E26" s="82"/>
-      <c r="F26" s="82"/>
-      <c r="G26" s="82"/>
+      <c r="B26" s="64"/>
+      <c r="C26" s="64"/>
+      <c r="D26" s="64"/>
+      <c r="E26" s="64"/>
+      <c r="F26" s="64"/>
+      <c r="G26" s="64"/>
     </row>
     <row r="27" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="18" t="s">
+      <c r="A27" s="15" t="s">
         <v>150</v>
       </c>
       <c r="B27" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C27" s="12" t="s">
+      <c r="C27" s="10" t="s">
         <v>151</v>
       </c>
-      <c r="D27" s="12" t="s">
+      <c r="D27" s="10" t="s">
         <v>137</v>
       </c>
-      <c r="E27" s="12" t="s">
+      <c r="E27" s="10" t="s">
         <v>138</v>
       </c>
-      <c r="F27" s="74" t="s">
+      <c r="F27" s="55" t="s">
         <v>152</v>
       </c>
-      <c r="G27" s="76" t="s">
+      <c r="G27" s="57" t="s">
         <v>153</v>
       </c>
     </row>
     <row r="28" spans="1:15" ht="15" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="16" t="s">
+      <c r="A28" s="13" t="s">
         <v>1</v>
       </c>
       <c r="B28" s="4">
@@ -2738,24 +2842,24 @@
         <v>1</v>
       </c>
       <c r="D28" s="2">
-        <f>N4</f>
+        <f t="shared" ref="D28:E30" si="1">N4</f>
         <v>1.02</v>
       </c>
       <c r="E28" s="2">
-        <f>O4</f>
+        <f t="shared" si="1"/>
         <v>0.875</v>
       </c>
-      <c r="F28" s="34">
+      <c r="F28" s="26">
         <f>$B$22</f>
         <v>2.0699999999999998</v>
       </c>
-      <c r="G28" s="77">
+      <c r="G28" s="58">
         <f>C28*(D28*E28*B28)/(F28^1.5)</f>
         <v>9.0589213101597383E-4</v>
       </c>
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A29" s="17" t="s">
+      <c r="A29" s="14" t="s">
         <v>154</v>
       </c>
       <c r="B29" s="3">
@@ -2766,24 +2870,24 @@
         <v>1</v>
       </c>
       <c r="D29" s="1">
-        <f>N5</f>
+        <f t="shared" si="1"/>
         <v>1.02</v>
       </c>
       <c r="E29" s="1">
-        <f>O5</f>
+        <f t="shared" si="1"/>
         <v>0.86250000000000004</v>
       </c>
-      <c r="F29" s="75">
-        <f t="shared" ref="F29:F34" si="1">$B$22</f>
+      <c r="F29" s="56">
+        <f t="shared" ref="F29:F34" si="2">$B$22</f>
         <v>2.0699999999999998</v>
       </c>
-      <c r="G29" s="37">
-        <f t="shared" ref="G29:G34" si="2">C29*(D29*E29*B29)/(F29^1.5)</f>
+      <c r="G29" s="29">
+        <f t="shared" ref="G29:G34" si="3">C29*(D29*E29*B29)/(F29^1.5)</f>
         <v>2.88040073958326E-4</v>
       </c>
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A30" s="17" t="s">
+      <c r="A30" s="14" t="s">
         <v>4</v>
       </c>
       <c r="B30" s="3">
@@ -2794,24 +2898,24 @@
         <v>1</v>
       </c>
       <c r="D30" s="1">
-        <f>N6</f>
+        <f t="shared" si="1"/>
         <v>1.03833</v>
       </c>
       <c r="E30" s="1">
-        <f>O6</f>
+        <f t="shared" si="1"/>
         <v>0.86199999999999999</v>
       </c>
-      <c r="F30" s="75">
-        <f t="shared" si="1"/>
+      <c r="F30" s="56">
+        <f t="shared" si="2"/>
         <v>2.0699999999999998</v>
       </c>
-      <c r="G30" s="37">
-        <f t="shared" si="2"/>
+      <c r="G30" s="29">
+        <f t="shared" si="3"/>
         <v>1.0656777073516555E-4</v>
       </c>
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A31" s="17" t="s">
+      <c r="A31" s="14" t="s">
         <v>2</v>
       </c>
       <c r="B31" s="3">
@@ -2829,17 +2933,17 @@
         <f>O8</f>
         <v>0.86250000000000004</v>
       </c>
-      <c r="F31" s="75">
-        <f t="shared" si="1"/>
+      <c r="F31" s="56">
+        <f t="shared" si="2"/>
         <v>2.0699999999999998</v>
       </c>
-      <c r="G31" s="37">
-        <f t="shared" si="2"/>
+      <c r="G31" s="29">
+        <f t="shared" si="3"/>
         <v>4.2332804856281391E-3</v>
       </c>
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A32" s="17" t="s">
+      <c r="A32" s="14" t="s">
         <v>155</v>
       </c>
       <c r="B32" s="3">
@@ -2857,17 +2961,17 @@
         <f>O9</f>
         <v>0.86250000000000004</v>
       </c>
-      <c r="F32" s="75">
-        <f t="shared" si="1"/>
+      <c r="F32" s="56">
+        <f t="shared" si="2"/>
         <v>2.0699999999999998</v>
       </c>
-      <c r="G32" s="37">
-        <f t="shared" si="2"/>
+      <c r="G32" s="29">
+        <f t="shared" si="3"/>
         <v>4.2818836316867371E-4</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A33" s="17" t="s">
+      <c r="A33" s="14" t="s">
         <v>5</v>
       </c>
       <c r="B33" s="3">
@@ -2885,17 +2989,17 @@
         <f>O11</f>
         <v>0.86250000000000004</v>
       </c>
-      <c r="F33" s="75">
-        <f t="shared" si="1"/>
+      <c r="F33" s="56">
+        <f t="shared" si="2"/>
         <v>2.0699999999999998</v>
       </c>
-      <c r="G33" s="37">
-        <f t="shared" si="2"/>
+      <c r="G33" s="29">
+        <f t="shared" si="3"/>
         <v>1.1244023936686617E-3</v>
       </c>
     </row>
     <row r="34" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="17" t="s">
+      <c r="A34" s="14" t="s">
         <v>6</v>
       </c>
       <c r="B34" s="3">
@@ -2913,26 +3017,33 @@
         <f>O12</f>
         <v>0.86250000000000004</v>
       </c>
-      <c r="F34" s="36">
-        <f t="shared" si="1"/>
+      <c r="F34" s="28">
+        <f t="shared" si="2"/>
         <v>2.0699999999999998</v>
       </c>
-      <c r="G34" s="85">
-        <f t="shared" si="2"/>
+      <c r="G34" s="60">
+        <f t="shared" si="3"/>
         <v>1.4306695234491047E-4</v>
       </c>
     </row>
     <row r="35" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="F35" s="86" t="s">
+      <c r="F35" s="61" t="s">
         <v>158</v>
       </c>
-      <c r="G35" s="87">
+      <c r="G35" s="62">
         <f>SUM(G28:G34)</f>
         <v>7.2294381705198503E-3</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="G37" s="73"/>
+    <row r="36" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="37" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="F37" s="79" t="s">
+        <v>161</v>
+      </c>
+      <c r="G37" s="80">
+        <f>G28+G31+G33+G34</f>
+        <v>6.4066419626576856E-3</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="14">
@@ -3170,6 +3281,134 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{78CBAC62-2666-4A5D-80B9-0D82AF074AF3}">
+  <dimension ref="A1:C13"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="16.44140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="2" spans="1:3" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="82" t="s">
+        <v>168</v>
+      </c>
+      <c r="B3" s="81"/>
+      <c r="C3" s="81"/>
+    </row>
+    <row r="4" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="B4" s="2">
+        <v>8.98</v>
+      </c>
+      <c r="C4" s="22" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="B5" s="1">
+        <v>0.2172</v>
+      </c>
+      <c r="C5" s="23" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="B6" s="1">
+        <v>0.16500000000000001</v>
+      </c>
+      <c r="C6" s="23" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="83" t="s">
+        <v>169</v>
+      </c>
+      <c r="B7" s="83"/>
+      <c r="C7" s="83"/>
+    </row>
+    <row r="8" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="B8" s="2">
+        <v>3.87</v>
+      </c>
+      <c r="C8" s="22" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="B9" s="1">
+        <v>8.5800000000000001E-2</v>
+      </c>
+      <c r="C9" s="23" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="B10" s="1">
+        <v>0.53500000000000003</v>
+      </c>
+      <c r="C10" s="23" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" s="84" t="s">
+        <v>172</v>
+      </c>
+      <c r="B12" s="85">
+        <f>((0.1*B4)/(B8+2))*0.8</f>
+        <v>0.12238500851788758</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="86" t="s">
+        <v>173</v>
+      </c>
+      <c r="B13" s="87">
+        <f>-((B9*B10)/(B5*B6))*B12</f>
+        <v>-0.15675648881066448</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A7:C7"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA935838-9803-4D28-BB5F-9527F2166E9C}">
   <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -3231,7 +3470,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E48C65C0-CE32-4736-962B-594A33BDB19E}">
   <dimension ref="A1:B19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -3397,7 +3636,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6CED5ACF-DC54-43BC-95C8-1A622F1EFA29}">
   <dimension ref="A1:B17"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -3547,7 +3786,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{168CB0EA-C8E2-45E5-AB6B-358E6234C580}">
   <dimension ref="A1:C8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -3627,7 +3866,7 @@
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" s="9" t="s">
+      <c r="A8" s="1" t="s">
         <v>122</v>
       </c>
       <c r="B8" s="1">
@@ -3642,23 +3881,23 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{390E4474-71C3-4371-935C-8F12FA2B8A53}">
   <dimension ref="A2:C26"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="2" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="26" t="s">
+      <c r="A2" s="72" t="s">
         <v>143</v>
       </c>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
+      <c r="B2" s="73"/>
+      <c r="C2" s="73"/>
     </row>
     <row r="3" spans="1:3" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="B3" s="20" t="s">
+      <c r="B3" s="17" t="s">
         <v>21</v>
       </c>
       <c r="C3" s="8" t="s">
@@ -3666,63 +3905,63 @@
       </c>
     </row>
     <row r="4" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="16" t="s">
+      <c r="A4" s="13" t="s">
         <v>144</v>
       </c>
       <c r="B4" s="4">
         <v>16.899999999999999</v>
       </c>
-      <c r="C4" s="30" t="s">
+      <c r="C4" s="22" t="s">
         <v>146</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="17" t="s">
+      <c r="A5" s="14" t="s">
         <v>145</v>
       </c>
       <c r="B5" s="3">
         <f>67.829</f>
         <v>67.828999999999994</v>
       </c>
-      <c r="C5" s="31" t="s">
+      <c r="C5" s="23" t="s">
         <v>146</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="17" t="s">
+      <c r="A6" s="14" t="s">
         <v>112</v>
       </c>
       <c r="B6" s="3">
         <f>B4/B5</f>
         <v>0.24915596573736898</v>
       </c>
-      <c r="C6" s="31" t="s">
+      <c r="C6" s="23" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="17" t="s">
+      <c r="A7" s="14" t="s">
         <v>8</v>
       </c>
       <c r="B7" s="3">
         <v>700</v>
       </c>
-      <c r="C7" s="31" t="s">
+      <c r="C7" s="23" t="s">
         <v>146</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="26" t="s">
+      <c r="A21" s="72" t="s">
         <v>148</v>
       </c>
-      <c r="B21" s="25"/>
-      <c r="C21" s="25"/>
+      <c r="B21" s="73"/>
+      <c r="C21" s="73"/>
     </row>
     <row r="22" spans="1:3" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A22" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="B22" s="20" t="s">
+      <c r="B22" s="17" t="s">
         <v>21</v>
       </c>
       <c r="C22" s="8" t="s">
@@ -3730,47 +3969,47 @@
       </c>
     </row>
     <row r="23" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="16" t="s">
+      <c r="A23" s="13" t="s">
         <v>144</v>
       </c>
       <c r="B23" s="4">
         <v>20</v>
       </c>
-      <c r="C23" s="30" t="s">
+      <c r="C23" s="22" t="s">
         <v>146</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A24" s="17" t="s">
+      <c r="A24" s="14" t="s">
         <v>145</v>
       </c>
       <c r="B24" s="3">
         <v>70</v>
       </c>
-      <c r="C24" s="31" t="s">
+      <c r="C24" s="23" t="s">
         <v>146</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A25" s="17" t="s">
+      <c r="A25" s="14" t="s">
         <v>112</v>
       </c>
       <c r="B25" s="3">
         <f>B23/B24</f>
         <v>0.2857142857142857</v>
       </c>
-      <c r="C25" s="31" t="s">
+      <c r="C25" s="23" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A26" s="17" t="s">
+      <c r="A26" s="14" t="s">
         <v>8</v>
       </c>
       <c r="B26" s="3">
         <v>610</v>
       </c>
-      <c r="C26" s="31" t="s">
+      <c r="C26" s="23" t="s">
         <v>146</v>
       </c>
     </row>

</xml_diff>